<commit_message>
extra scenario with load
</commit_message>
<xml_diff>
--- a/examples/scripts/test_pv.xlsx
+++ b/examples/scripts/test_pv.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\FS01\RedirectedFolders\Max.Libberoth\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Max.Libberoth\PycharmProjects\oemof-tabular-plugins\examples\scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="78">
   <si>
     <t>dispatchable</t>
   </si>
@@ -246,6 +246,18 @@
   </si>
   <si>
     <t>pv_capacity 0.11 kW, 239 kWh annually….1770 kWh/kWp in Morocco (1600-1700 reference)</t>
+  </si>
+  <si>
+    <t>test_pv_load_8</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> pv_capacity 0.04 kW</t>
+  </si>
+  <si>
+    <t>ghi*pv_efficiency_gni*modules_per_m2*ghi_to_gni</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> pv_capacity 0.04 kW, excess marginal_cost must not outnumber back-up-elec marginal_cost (if so, simulation will be unbounded)</t>
   </si>
 </sst>
 </file>
@@ -687,7 +699,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S56"/>
+  <dimension ref="A1:S61"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.08984375" customWidth="1"/>
@@ -2830,6 +2842,210 @@
         <v>73</v>
       </c>
     </row>
+    <row r="57" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A57" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B57" s="1"/>
+      <c r="C57" s="2"/>
+      <c r="D57" s="2"/>
+      <c r="E57" s="2"/>
+      <c r="F57" s="1">
+        <v>0</v>
+      </c>
+      <c r="G57">
+        <v>1</v>
+      </c>
+      <c r="H57" t="s">
+        <v>20</v>
+      </c>
+      <c r="I57" t="s">
+        <v>10</v>
+      </c>
+      <c r="J57" s="1">
+        <v>1</v>
+      </c>
+      <c r="L57" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="M57" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="N57" s="2">
+        <v>1</v>
+      </c>
+      <c r="O57" t="s">
+        <v>69</v>
+      </c>
+      <c r="P57" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q57" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="R57" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="S57" s="13" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="58" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A58" s="10"/>
+      <c r="B58" s="11"/>
+      <c r="C58" s="9"/>
+      <c r="D58" s="9"/>
+      <c r="E58" s="9"/>
+      <c r="F58" s="11"/>
+      <c r="G58" s="9"/>
+      <c r="H58" s="9"/>
+      <c r="I58" s="9"/>
+      <c r="J58" s="11"/>
+      <c r="K58" s="10"/>
+      <c r="L58" s="10"/>
+      <c r="M58" s="10"/>
+      <c r="N58" s="10"/>
+      <c r="O58" s="12"/>
+      <c r="P58" s="10"/>
+      <c r="Q58" s="10"/>
+      <c r="R58" s="9"/>
+      <c r="S58" s="9"/>
+    </row>
+    <row r="59" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A59" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C59" s="3"/>
+      <c r="D59" s="3"/>
+      <c r="E59" s="3"/>
+      <c r="F59" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G59" s="3"/>
+      <c r="H59" s="3"/>
+      <c r="I59" s="3"/>
+      <c r="J59" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="K59" s="3"/>
+      <c r="L59" s="3"/>
+      <c r="M59" s="3"/>
+      <c r="N59" s="3"/>
+      <c r="O59" s="8"/>
+      <c r="P59" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q59" s="3"/>
+      <c r="R59" s="3"/>
+      <c r="S59" s="3"/>
+    </row>
+    <row r="60" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A60" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="B60" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C60" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="D60" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="E60" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="F60" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="G60" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="H60" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="I60" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="J60" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="K60" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="L60" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="M60" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="N60" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="O60" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="P60" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q60" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="R60" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="S60" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="61" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A61" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="B61" s="1"/>
+      <c r="F61" s="1">
+        <v>0</v>
+      </c>
+      <c r="G61">
+        <v>1</v>
+      </c>
+      <c r="H61" t="s">
+        <v>20</v>
+      </c>
+      <c r="I61" t="s">
+        <v>10</v>
+      </c>
+      <c r="J61" s="1">
+        <v>0</v>
+      </c>
+      <c r="L61" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="M61" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="N61" s="2">
+        <v>1</v>
+      </c>
+      <c r="O61" t="s">
+        <v>69</v>
+      </c>
+      <c r="P61" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q61" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="R61" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="S61" s="13" t="s">
+        <v>77</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
extra test scenario, better results documentation
</commit_message>
<xml_diff>
--- a/examples/scripts/test_pv.xlsx
+++ b/examples/scripts/test_pv.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="94">
   <si>
     <t>dispatchable</t>
   </si>
@@ -89,9 +89,6 @@
     <t>ghi-profile</t>
   </si>
   <si>
-    <t>comment</t>
-  </si>
-  <si>
     <t>infeasible</t>
   </si>
   <si>
@@ -188,9 +185,6 @@
     <t>pv_capacity in m2, pv output in kW, PROBLEM IF output higher than 1 kW/m2</t>
   </si>
   <si>
-    <t>pv_capacity 0.05 [?kW?], pv output in kW (not peak capacity, but maximum output of test profiles as optimized capacity)</t>
-  </si>
-  <si>
     <t>_volpot_pvopen_belfaa</t>
   </si>
   <si>
@@ -203,12 +197,6 @@
     <t>ghi*pv_efficiency*modules_per_m4</t>
   </si>
   <si>
-    <t>same as before but updatet PV module parameters, pv_capacity 0.13 kW (should be 0.135 kWp), 273 kWh annually, 2020 kWh/kWp (still a little high but better)</t>
-  </si>
-  <si>
-    <t>pv_capacity 0.16 ?kW?, 334 kWh annually, ~0.3 modules per m2 with 450 Wp results in 0.135 kWp (lower than peak production of 0.16) and 2480 kWh/kWp (morocco expectation 1600-1700)</t>
-  </si>
-  <si>
     <t>test_pv_noload_7</t>
   </si>
   <si>
@@ -239,32 +227,92 @@
     <t>ghi*pv_efficiency_gni*modules_per_m2 / ghi_to_gni</t>
   </si>
   <si>
-    <t>ghi*pv_efficiency_gni*modules_per_m3*ghi_to_gni</t>
-  </si>
-  <si>
-    <t>irradiation perpendicular to PV module (Global normal irradiance GNI) with ghi_to_gni =  cos(tilt) used, 0.15 kW pv_capacity and 318 kWh too high</t>
-  </si>
-  <si>
-    <t>pv_capacity 0.11 kW, 239 kWh annually….1770 kWh/kWp in Morocco (1600-1700 reference)</t>
-  </si>
-  <si>
     <t>test_pv_load_8</t>
   </si>
   <si>
-    <t xml:space="preserve"> pv_capacity 0.04 kW</t>
-  </si>
-  <si>
     <t>ghi*pv_efficiency_gni*modules_per_m2*ghi_to_gni</t>
   </si>
   <si>
-    <t xml:space="preserve"> pv_capacity 0.04 kW, excess marginal_cost must not outnumber back-up-elec marginal_cost (if so, simulation will be unbounded)</t>
+    <t>for source output can be higher than capacity (300 W on 1 m2), for converter this seems not possible</t>
+  </si>
+  <si>
+    <t>evaluation</t>
+  </si>
+  <si>
+    <t>elec_profile should be ghi*pv_efficiency</t>
+  </si>
+  <si>
+    <t>solar_capacity</t>
+  </si>
+  <si>
+    <t>pv_capacity</t>
+  </si>
+  <si>
+    <t>pv_total_output</t>
+  </si>
+  <si>
+    <t>0.05 kW</t>
+  </si>
+  <si>
+    <t>1 m2</t>
+  </si>
+  <si>
+    <t>0.16 kW</t>
+  </si>
+  <si>
+    <t>0.13 kW</t>
+  </si>
+  <si>
+    <t>273 kWh</t>
+  </si>
+  <si>
+    <t>pv_capacity not peak capacity, but maximum pv output of test profiles [kW]</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ~0.3 modules per m2 with 450 Wp results in 0.135 kWp (lower than peak production of 0.16) and 2480 kWh/kWp (morocco expectation 1600-1700)</t>
+  </si>
+  <si>
+    <t>updatet PV module parameters, pv_capacity 0.13 kW (should be 0.135 kWp), 2020 kWh/kWp (still a little high but better)</t>
+  </si>
+  <si>
+    <t>0.15 kW</t>
+  </si>
+  <si>
+    <t>318 kWh</t>
+  </si>
+  <si>
+    <t>irradiation perpendicular to PV module (Global normal irradiance GNI) with GNI = GHI*cos(tilt) = GHI*ghi_to_gni; pv_capacity and output too high</t>
+  </si>
+  <si>
+    <t>239 kWh</t>
+  </si>
+  <si>
+    <t>0.11 kW</t>
+  </si>
+  <si>
+    <t>0.04 kW</t>
+  </si>
+  <si>
+    <t>334 kWh</t>
+  </si>
+  <si>
+    <t>optimization will be unbounded if excess marginal_cost higher than back-up-elec marginal_cost (in absolute numbers)</t>
+  </si>
+  <si>
+    <t>1770 kWh/kWp in Morocco (1600-1700 reference), but pv peak capacity is 0.135 kWp</t>
+  </si>
+  <si>
+    <t>pv_capacity can be linked to solar_cap via Constraint; this approach will lead to problems if pv_output is higher than 1 kW/m2 at any time step</t>
+  </si>
+  <si>
+    <t>pv_capacity below real peak capacity of 0.135 kWp, but real peak capacity could be accessed separately</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -279,8 +327,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -292,8 +354,18 @@
         <fgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -390,12 +462,25 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
@@ -413,14 +498,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="3"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="3" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="4">
     <cellStyle name="Gut" xfId="1" builtinId="26"/>
+    <cellStyle name="Neutral" xfId="3" builtinId="28"/>
+    <cellStyle name="Schlecht" xfId="2" builtinId="27"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -699,7 +788,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S61"/>
+  <dimension ref="A1:V62"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.08984375" customWidth="1"/>
@@ -709,9 +798,12 @@
     <col min="15" max="15" width="13.7265625" customWidth="1"/>
     <col min="17" max="17" width="17.81640625" customWidth="1"/>
     <col min="18" max="18" width="25.6328125" customWidth="1"/>
+    <col min="19" max="19" width="11.36328125" customWidth="1"/>
+    <col min="20" max="20" width="10" customWidth="1"/>
+    <col min="21" max="21" width="11.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>7</v>
       </c>
@@ -733,9 +825,9 @@
       </c>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>1</v>
@@ -771,28 +863,37 @@
         <v>4</v>
       </c>
       <c r="M2" s="9" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="N2" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="O2" s="7" t="s">
         <v>28</v>
-      </c>
-      <c r="O2" s="7" t="s">
-        <v>29</v>
       </c>
       <c r="P2" s="6" t="s">
         <v>16</v>
       </c>
       <c r="Q2" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R2" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="S2" s="6" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.35">
+        <v>72</v>
+      </c>
+      <c r="T2" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="U2" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="V2" s="6" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="3" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>11</v>
       </c>
@@ -818,7 +919,7 @@
         <v>9</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="N3" s="2">
         <v>1</v>
@@ -830,13 +931,14 @@
         <v>17</v>
       </c>
       <c r="Q3" t="s">
+        <v>29</v>
+      </c>
+      <c r="R3" t="s">
         <v>30</v>
       </c>
-      <c r="R3" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="V3" s="20"/>
+    </row>
+    <row r="4" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>12</v>
       </c>
@@ -860,7 +962,7 @@
         <v>9</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="N4" s="2">
         <v>1</v>
@@ -872,13 +974,14 @@
         <v>17</v>
       </c>
       <c r="Q4" t="s">
+        <v>29</v>
+      </c>
+      <c r="R4" t="s">
         <v>30</v>
       </c>
-      <c r="R4" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="V4" s="20"/>
+    </row>
+    <row r="5" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
         <v>13</v>
       </c>
@@ -903,7 +1006,7 @@
         <v>10</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="N5" s="2">
         <v>1</v>
@@ -915,13 +1018,14 @@
         <v>17</v>
       </c>
       <c r="Q5" t="s">
+        <v>29</v>
+      </c>
+      <c r="R5" t="s">
         <v>30</v>
       </c>
-      <c r="R5" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="V5" s="20"/>
+    </row>
+    <row r="6" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
         <v>14</v>
       </c>
@@ -948,7 +1052,7 @@
         <v>10</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="N6" s="2">
         <v>1</v>
@@ -960,13 +1064,14 @@
         <v>17</v>
       </c>
       <c r="Q6" t="s">
+        <v>29</v>
+      </c>
+      <c r="R6" t="s">
         <v>30</v>
       </c>
-      <c r="R6" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="V6" s="20"/>
+    </row>
+    <row r="7" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
         <v>18</v>
       </c>
@@ -990,7 +1095,7 @@
         <v>9</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="N7" s="2">
         <v>1</v>
@@ -999,15 +1104,18 @@
         <v>0.5</v>
       </c>
       <c r="P7" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q7" s="5"/>
       <c r="R7" s="5"/>
-      <c r="S7" s="5" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="S7" s="5"/>
+      <c r="T7" s="5"/>
+      <c r="U7" s="5"/>
+      <c r="V7" s="21" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
         <v>19</v>
       </c>
@@ -1034,7 +1142,7 @@
         <v>10</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="N8" s="2">
         <v>1</v>
@@ -1043,16 +1151,16 @@
         <v>0.5</v>
       </c>
       <c r="P8" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="Q8" s="5"/>
+      <c r="V8" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="Q8" s="5"/>
-      <c r="S8" t="s">
+    </row>
+    <row r="9" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A9" s="5" t="s">
         <v>23</v>
-      </c>
-    </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A9" s="5" t="s">
-        <v>24</v>
       </c>
       <c r="B9" s="1"/>
       <c r="C9" s="2"/>
@@ -1077,7 +1185,7 @@
         <v>9</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="N9" s="2">
         <v>1</v>
@@ -1089,15 +1197,19 @@
         <v>17</v>
       </c>
       <c r="Q9" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="R9" s="5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.35">
+        <v>31</v>
+      </c>
+      <c r="S9" s="5"/>
+      <c r="T9" s="5"/>
+      <c r="U9" s="5"/>
+      <c r="V9" s="20"/>
+    </row>
+    <row r="10" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B10" s="1"/>
       <c r="C10" s="2"/>
@@ -1125,7 +1237,7 @@
         <v>10</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="N10" s="2">
         <v>1</v>
@@ -1137,15 +1249,19 @@
         <v>17</v>
       </c>
       <c r="Q10" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="R10" s="5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.35">
+        <v>31</v>
+      </c>
+      <c r="S10" s="5"/>
+      <c r="T10" s="5"/>
+      <c r="U10" s="5"/>
+      <c r="V10" s="20"/>
+    </row>
+    <row r="11" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A11" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B11" s="1"/>
       <c r="C11" s="2"/>
@@ -1173,8 +1289,14 @@
         <v>20</v>
       </c>
       <c r="R11" s="5"/>
-    </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="S11" s="5"/>
+      <c r="T11" s="5"/>
+      <c r="U11" s="5"/>
+      <c r="V11" s="19" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="12" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A12" s="5"/>
       <c r="B12" s="1"/>
       <c r="C12" s="2"/>
@@ -1190,8 +1312,11 @@
       <c r="P12" s="5"/>
       <c r="Q12" s="5"/>
       <c r="R12" s="5"/>
-    </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="S12" s="5"/>
+      <c r="T12" s="5"/>
+      <c r="U12" s="5"/>
+    </row>
+    <row r="13" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A13" s="10"/>
       <c r="B13" s="11"/>
       <c r="C13" s="9"/>
@@ -1211,8 +1336,11 @@
       <c r="Q13" s="10"/>
       <c r="R13" s="9"/>
       <c r="S13" s="9"/>
-    </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="T13" s="9"/>
+      <c r="U13" s="9"/>
+      <c r="V13" s="9"/>
+    </row>
+    <row r="14" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>7</v>
       </c>
@@ -1234,9 +1362,9 @@
       </c>
       <c r="Q14" s="2"/>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>1</v>
@@ -1272,28 +1400,37 @@
         <v>4</v>
       </c>
       <c r="M15" s="9" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="N15" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="O15" s="12" t="s">
         <v>28</v>
-      </c>
-      <c r="O15" s="12" t="s">
-        <v>29</v>
       </c>
       <c r="P15" s="6" t="s">
         <v>16</v>
       </c>
       <c r="Q15" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R15" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="S15" s="6" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.35">
+        <v>72</v>
+      </c>
+      <c r="T15" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="U15" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="V15" s="6" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="16" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
         <v>11</v>
       </c>
@@ -1319,25 +1456,26 @@
         <v>9</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="N16" s="2">
         <v>1</v>
       </c>
       <c r="O16" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="P16" s="2" t="s">
         <v>17</v>
       </c>
       <c r="Q16" s="13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="R16" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.35">
+        <v>30</v>
+      </c>
+      <c r="V16" s="20"/>
+    </row>
+    <row r="17" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A17" s="5" t="s">
         <v>18</v>
       </c>
@@ -1361,24 +1499,27 @@
         <v>9</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="N17" s="2">
         <v>1</v>
       </c>
       <c r="O17" s="7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="P17" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q17" s="5"/>
       <c r="R17" s="5"/>
       <c r="S17" s="5"/>
-    </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="T17" s="5"/>
+      <c r="U17" s="5"/>
+      <c r="V17" s="21"/>
+    </row>
+    <row r="18" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A18" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B18" s="1"/>
       <c r="C18" s="2"/>
@@ -1403,27 +1544,31 @@
         <v>9</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="N18" s="2">
         <v>1</v>
       </c>
       <c r="O18" s="7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="P18" s="5" t="s">
         <v>17</v>
       </c>
       <c r="Q18" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="R18" s="5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.35">
+        <v>31</v>
+      </c>
+      <c r="S18" s="5"/>
+      <c r="T18" s="5"/>
+      <c r="U18" s="5"/>
+      <c r="V18" s="20"/>
+    </row>
+    <row r="19" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A19" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B19" s="1"/>
       <c r="C19" s="2"/>
@@ -1448,13 +1593,13 @@
         <v>10</v>
       </c>
       <c r="M19" s="2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="N19" s="5">
         <v>1</v>
       </c>
       <c r="O19" s="7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="P19" s="5" t="s">
         <v>17</v>
@@ -1463,13 +1608,16 @@
         <v>8</v>
       </c>
       <c r="R19" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="S19" s="5"/>
+      <c r="T19" s="5"/>
+      <c r="U19" s="5"/>
+      <c r="V19" s="22" t="s">
         <v>49</v>
       </c>
-      <c r="S19" s="5" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.35">
+    </row>
+    <row r="20" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A20" s="5"/>
       <c r="B20" s="1"/>
       <c r="C20" s="2"/>
@@ -1484,8 +1632,11 @@
       <c r="P20" s="5"/>
       <c r="Q20" s="5"/>
       <c r="R20" s="5"/>
-    </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="S20" s="5"/>
+      <c r="T20" s="5"/>
+      <c r="U20" s="5"/>
+    </row>
+    <row r="21" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A21" s="10"/>
       <c r="B21" s="11"/>
       <c r="C21" s="9"/>
@@ -1505,8 +1656,11 @@
       <c r="Q21" s="10"/>
       <c r="R21" s="9"/>
       <c r="S21" s="9"/>
-    </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="T21" s="9"/>
+      <c r="U21" s="9"/>
+      <c r="V21" s="9"/>
+    </row>
+    <row r="22" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>7</v>
       </c>
@@ -1528,9 +1682,9 @@
       </c>
       <c r="Q22" s="2"/>
     </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>1</v>
@@ -1566,28 +1720,37 @@
         <v>4</v>
       </c>
       <c r="M23" s="9" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="N23" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="O23" s="12" t="s">
         <v>28</v>
-      </c>
-      <c r="O23" s="12" t="s">
-        <v>29</v>
       </c>
       <c r="P23" s="6" t="s">
         <v>16</v>
       </c>
       <c r="Q23" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R23" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="S23" s="6" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.35">
+        <v>72</v>
+      </c>
+      <c r="T23" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="U23" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="V23" s="6" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="24" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
         <v>11</v>
       </c>
@@ -1613,13 +1776,13 @@
         <v>9</v>
       </c>
       <c r="M24" s="2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="N24" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="O24" s="7" t="s">
         <v>38</v>
-      </c>
-      <c r="O24" s="7" t="s">
-        <v>39</v>
       </c>
       <c r="P24" s="2" t="s">
         <v>17</v>
@@ -1628,10 +1791,13 @@
         <v>20</v>
       </c>
       <c r="R24" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.35">
+        <v>38</v>
+      </c>
+      <c r="V24" s="20" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="25" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A25" s="5" t="s">
         <v>18</v>
       </c>
@@ -1655,13 +1821,13 @@
         <v>9</v>
       </c>
       <c r="M25" s="2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="N25" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="O25" s="7" t="s">
         <v>38</v>
-      </c>
-      <c r="O25" s="7" t="s">
-        <v>39</v>
       </c>
       <c r="P25" s="5" t="s">
         <v>17</v>
@@ -1670,13 +1836,16 @@
         <v>20</v>
       </c>
       <c r="R25" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="S25" s="5"/>
-    </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.35">
+        <v>38</v>
+      </c>
+      <c r="S25" s="13"/>
+      <c r="T25" s="13"/>
+      <c r="U25" s="13"/>
+      <c r="V25" s="21"/>
+    </row>
+    <row r="26" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A26" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B26" s="1"/>
       <c r="C26" s="2"/>
@@ -1701,13 +1870,13 @@
         <v>9</v>
       </c>
       <c r="M26" s="2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="N26" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="O26" s="7" t="s">
         <v>38</v>
-      </c>
-      <c r="O26" s="7" t="s">
-        <v>39</v>
       </c>
       <c r="P26" s="5" t="s">
         <v>17</v>
@@ -1716,10 +1885,14 @@
         <v>20</v>
       </c>
       <c r="R26" s="5" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.35">
+        <v>38</v>
+      </c>
+      <c r="S26" s="5"/>
+      <c r="T26" s="5"/>
+      <c r="U26" s="5"/>
+      <c r="V26" s="20"/>
+    </row>
+    <row r="27" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A27" s="5"/>
       <c r="B27" s="1"/>
       <c r="C27" s="2"/>
@@ -1734,8 +1907,11 @@
       <c r="P27" s="5"/>
       <c r="Q27" s="5"/>
       <c r="R27" s="5"/>
-    </row>
-    <row r="28" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="S27" s="5"/>
+      <c r="T27" s="5"/>
+      <c r="U27" s="5"/>
+    </row>
+    <row r="28" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A28" s="10"/>
       <c r="B28" s="11"/>
       <c r="C28" s="9"/>
@@ -1755,8 +1931,11 @@
       <c r="Q28" s="10"/>
       <c r="R28" s="9"/>
       <c r="S28" s="9"/>
-    </row>
-    <row r="29" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="T28" s="9"/>
+      <c r="U28" s="9"/>
+      <c r="V28" s="9"/>
+    </row>
+    <row r="29" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>7</v>
       </c>
@@ -1778,9 +1957,9 @@
       </c>
       <c r="Q29" s="2"/>
     </row>
-    <row r="30" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>1</v>
@@ -1816,28 +1995,37 @@
         <v>4</v>
       </c>
       <c r="M30" s="9" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="N30" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="O30" s="12" t="s">
         <v>28</v>
-      </c>
-      <c r="O30" s="12" t="s">
-        <v>29</v>
       </c>
       <c r="P30" s="6" t="s">
         <v>16</v>
       </c>
       <c r="Q30" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R30" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="S30" s="6" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="31" spans="1:19" x14ac:dyDescent="0.35">
+        <v>72</v>
+      </c>
+      <c r="T30" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="U30" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="V30" s="6" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="31" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A31" s="3" t="s">
         <v>11</v>
       </c>
@@ -1863,25 +2051,26 @@
         <v>9</v>
       </c>
       <c r="M31" s="2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="N31" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="O31" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="P31" s="2" t="s">
         <v>17</v>
       </c>
       <c r="Q31" s="13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="R31" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="32" spans="1:19" x14ac:dyDescent="0.35">
+        <v>30</v>
+      </c>
+      <c r="V31" s="20"/>
+    </row>
+    <row r="32" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A32" s="5" t="s">
         <v>18</v>
       </c>
@@ -1905,24 +2094,27 @@
         <v>9</v>
       </c>
       <c r="M32" s="2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="N32" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="O32" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="P32" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q32" s="13"/>
       <c r="R32" s="13"/>
-      <c r="S32" s="5"/>
-    </row>
-    <row r="33" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="S32" s="13"/>
+      <c r="T32" s="13"/>
+      <c r="U32" s="13"/>
+      <c r="V32" s="21"/>
+    </row>
+    <row r="33" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A33" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B33" s="1"/>
       <c r="C33" s="2"/>
@@ -1947,25 +2139,29 @@
         <v>9</v>
       </c>
       <c r="M33" s="2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="N33" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="O33" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="P33" s="5" t="s">
         <v>17</v>
       </c>
       <c r="Q33" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="R33" s="5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="34" spans="1:19" x14ac:dyDescent="0.35">
+        <v>31</v>
+      </c>
+      <c r="S33" s="5"/>
+      <c r="T33" s="5"/>
+      <c r="U33" s="5"/>
+      <c r="V33" s="20"/>
+    </row>
+    <row r="34" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A34" s="5"/>
       <c r="B34" s="1"/>
       <c r="C34" s="2"/>
@@ -1980,8 +2176,11 @@
       <c r="P34" s="5"/>
       <c r="Q34" s="5"/>
       <c r="R34" s="5"/>
-    </row>
-    <row r="35" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="S34" s="5"/>
+      <c r="T34" s="5"/>
+      <c r="U34" s="5"/>
+    </row>
+    <row r="35" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A35" s="10"/>
       <c r="B35" s="11"/>
       <c r="C35" s="9"/>
@@ -2001,8 +2200,11 @@
       <c r="Q35" s="10"/>
       <c r="R35" s="9"/>
       <c r="S35" s="9"/>
-    </row>
-    <row r="36" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="T35" s="9"/>
+      <c r="U35" s="9"/>
+      <c r="V35" s="9"/>
+    </row>
+    <row r="36" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>7</v>
       </c>
@@ -2024,9 +2226,9 @@
       </c>
       <c r="Q36" s="2"/>
     </row>
-    <row r="37" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>1</v>
@@ -2062,28 +2264,37 @@
         <v>4</v>
       </c>
       <c r="M37" s="9" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="N37" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="O37" s="12" t="s">
         <v>28</v>
-      </c>
-      <c r="O37" s="12" t="s">
-        <v>29</v>
       </c>
       <c r="P37" s="6" t="s">
         <v>16</v>
       </c>
       <c r="Q37" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R37" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="S37" s="6" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="38" spans="1:19" x14ac:dyDescent="0.35">
+        <v>72</v>
+      </c>
+      <c r="T37" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="U37" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="V37" s="6" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="38" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A38" s="3" t="s">
         <v>11</v>
       </c>
@@ -2109,25 +2320,26 @@
         <v>9</v>
       </c>
       <c r="M38" s="2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="N38" s="2">
         <v>1</v>
       </c>
       <c r="O38" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="P38" s="2" t="s">
         <v>17</v>
       </c>
       <c r="Q38" s="13" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="R38" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="39" spans="1:19" x14ac:dyDescent="0.35">
+        <v>30</v>
+      </c>
+      <c r="V38" s="20"/>
+    </row>
+    <row r="39" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A39" s="5" t="s">
         <v>18</v>
       </c>
@@ -2151,24 +2363,27 @@
         <v>9</v>
       </c>
       <c r="M39" s="2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="N39" s="2">
         <v>1</v>
       </c>
       <c r="O39" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="P39" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q39" s="13"/>
       <c r="R39" s="13"/>
-      <c r="S39" s="5"/>
-    </row>
-    <row r="40" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="S39" s="13"/>
+      <c r="T39" s="13"/>
+      <c r="U39" s="13"/>
+      <c r="V39" s="21"/>
+    </row>
+    <row r="40" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A40" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B40" s="1"/>
       <c r="C40" s="2"/>
@@ -2193,25 +2408,29 @@
         <v>9</v>
       </c>
       <c r="M40" s="2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="N40" s="2">
         <v>1</v>
       </c>
       <c r="O40" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="P40" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="Q40" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="R40" s="5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="41" spans="1:19" x14ac:dyDescent="0.35">
+        <v>31</v>
+      </c>
+      <c r="S40" s="5"/>
+      <c r="T40" s="5"/>
+      <c r="U40" s="5"/>
+      <c r="V40" s="20"/>
+    </row>
+    <row r="41" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A41" s="5"/>
       <c r="B41" s="1"/>
       <c r="C41" s="2"/>
@@ -2226,8 +2445,11 @@
       <c r="P41" s="5"/>
       <c r="Q41" s="5"/>
       <c r="R41" s="5"/>
-    </row>
-    <row r="42" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="S41" s="5"/>
+      <c r="T41" s="5"/>
+      <c r="U41" s="5"/>
+    </row>
+    <row r="42" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A42" s="10"/>
       <c r="B42" s="11"/>
       <c r="C42" s="9"/>
@@ -2247,8 +2469,11 @@
       <c r="Q42" s="10"/>
       <c r="R42" s="9"/>
       <c r="S42" s="9"/>
-    </row>
-    <row r="43" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="T42" s="9"/>
+      <c r="U42" s="9"/>
+      <c r="V42" s="9"/>
+    </row>
+    <row r="43" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A43" s="3" t="s">
         <v>7</v>
       </c>
@@ -2278,10 +2503,13 @@
       <c r="Q43" s="3"/>
       <c r="R43" s="3"/>
       <c r="S43" s="3"/>
-    </row>
-    <row r="44" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="T43" s="3"/>
+      <c r="U43" s="3"/>
+      <c r="V43" s="3"/>
+    </row>
+    <row r="44" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A44" s="9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B44" s="11" t="s">
         <v>1</v>
@@ -2317,30 +2545,39 @@
         <v>4</v>
       </c>
       <c r="M44" s="9" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="N44" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="O44" s="12" t="s">
         <v>28</v>
-      </c>
-      <c r="O44" s="12" t="s">
-        <v>29</v>
       </c>
       <c r="P44" s="6" t="s">
         <v>16</v>
       </c>
       <c r="Q44" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R44" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="S44" s="6" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="45" spans="1:19" x14ac:dyDescent="0.35">
+        <v>72</v>
+      </c>
+      <c r="T44" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="U44" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="V44" s="6" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="45" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A45" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B45" s="1"/>
       <c r="C45" s="2"/>
@@ -2365,13 +2602,13 @@
         <v>10</v>
       </c>
       <c r="M45" s="2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="N45" s="2">
         <v>1</v>
       </c>
       <c r="O45" s="15" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="P45" s="2" t="s">
         <v>17</v>
@@ -2380,15 +2617,22 @@
         <v>20</v>
       </c>
       <c r="R45" s="13" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="S45" s="13" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="46" spans="1:19" x14ac:dyDescent="0.35">
+        <v>76</v>
+      </c>
+      <c r="T45" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="U45" s="13"/>
+      <c r="V45" s="22" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="46" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A46" s="14" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B46" s="1"/>
       <c r="C46" s="2"/>
@@ -2413,13 +2657,13 @@
         <v>9</v>
       </c>
       <c r="M46" s="2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="N46" s="2">
         <v>1</v>
       </c>
       <c r="O46" s="16" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="P46" s="5" t="s">
         <v>17</v>
@@ -2428,15 +2672,22 @@
         <v>20</v>
       </c>
       <c r="R46" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="S46" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="T46" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="U46" s="13"/>
+      <c r="V46" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="S46" s="13" t="s">
+    </row>
+    <row r="47" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A47" s="14" t="s">
         <v>53</v>
-      </c>
-    </row>
-    <row r="47" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A47" s="14" t="s">
-        <v>55</v>
       </c>
       <c r="B47" s="1"/>
       <c r="C47" s="2"/>
@@ -2461,13 +2712,13 @@
         <v>10</v>
       </c>
       <c r="M47" s="2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="N47" s="2">
         <v>1</v>
       </c>
       <c r="O47" s="16" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="P47" s="5" t="s">
         <v>17</v>
@@ -2476,15 +2727,24 @@
         <v>20</v>
       </c>
       <c r="R47" s="13" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="S47" s="13" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="48" spans="1:19" x14ac:dyDescent="0.35">
+        <v>76</v>
+      </c>
+      <c r="T47" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="U47" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="V47" s="22" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="48" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A48" s="5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B48" s="1"/>
       <c r="C48" s="2"/>
@@ -2509,13 +2769,13 @@
         <v>10</v>
       </c>
       <c r="M48" s="2" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="N48" s="2">
         <v>1</v>
       </c>
       <c r="O48" s="16" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="P48" s="5" t="s">
         <v>17</v>
@@ -2524,13 +2784,22 @@
         <v>20</v>
       </c>
       <c r="R48" s="13" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="S48" s="13" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="49" spans="1:19" x14ac:dyDescent="0.35">
+        <v>76</v>
+      </c>
+      <c r="T48" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="U48" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="V48" s="22" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="49" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A49" s="10"/>
       <c r="B49" s="11"/>
       <c r="C49" s="9"/>
@@ -2550,8 +2819,11 @@
       <c r="Q49" s="10"/>
       <c r="R49" s="9"/>
       <c r="S49" s="9"/>
-    </row>
-    <row r="50" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="T49" s="9"/>
+      <c r="U49" s="9"/>
+      <c r="V49" s="9"/>
+    </row>
+    <row r="50" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A50" s="3" t="s">
         <v>7</v>
       </c>
@@ -2581,10 +2853,13 @@
       <c r="Q50" s="3"/>
       <c r="R50" s="3"/>
       <c r="S50" s="3"/>
-    </row>
-    <row r="51" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="T50" s="3"/>
+      <c r="U50" s="3"/>
+      <c r="V50" s="3"/>
+    </row>
+    <row r="51" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A51" s="9" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="B51" s="11" t="s">
         <v>1</v>
@@ -2620,30 +2895,39 @@
         <v>4</v>
       </c>
       <c r="M51" s="9" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="N51" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="O51" s="12" t="s">
         <v>28</v>
-      </c>
-      <c r="O51" s="12" t="s">
-        <v>29</v>
       </c>
       <c r="P51" s="6" t="s">
         <v>16</v>
       </c>
       <c r="Q51" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R51" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="S51" s="6" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="52" spans="1:19" x14ac:dyDescent="0.35">
+        <v>72</v>
+      </c>
+      <c r="T51" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="U51" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="V51" s="6" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="52" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A52" s="14" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B52" s="1"/>
       <c r="F52" s="1">
@@ -2665,13 +2949,13 @@
         <v>10</v>
       </c>
       <c r="M52" s="2" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="N52" s="2" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="O52" s="16" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="P52" s="5" t="s">
         <v>17</v>
@@ -2680,13 +2964,22 @@
         <v>20</v>
       </c>
       <c r="R52" s="13" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="S52" s="13" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="53" spans="1:19" x14ac:dyDescent="0.35">
+        <v>76</v>
+      </c>
+      <c r="T52" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="U52" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="V52" s="22" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="53" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A53" s="10"/>
       <c r="B53" s="11"/>
       <c r="C53" s="9"/>
@@ -2706,8 +2999,11 @@
       <c r="Q53" s="10"/>
       <c r="R53" s="9"/>
       <c r="S53" s="9"/>
-    </row>
-    <row r="54" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="T53" s="9"/>
+      <c r="U53" s="9"/>
+      <c r="V53" s="9"/>
+    </row>
+    <row r="54" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A54" s="3" t="s">
         <v>7</v>
       </c>
@@ -2737,10 +3033,13 @@
       <c r="Q54" s="3"/>
       <c r="R54" s="3"/>
       <c r="S54" s="3"/>
-    </row>
-    <row r="55" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="T54" s="3"/>
+      <c r="U54" s="3"/>
+      <c r="V54" s="3"/>
+    </row>
+    <row r="55" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A55" s="9" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="B55" s="11" t="s">
         <v>1</v>
@@ -2776,75 +3075,93 @@
         <v>4</v>
       </c>
       <c r="M55" s="9" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="N55" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="O55" s="12" t="s">
         <v>28</v>
-      </c>
-      <c r="O55" s="12" t="s">
-        <v>29</v>
       </c>
       <c r="P55" s="6" t="s">
         <v>16</v>
       </c>
       <c r="Q55" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R55" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="S55" s="6" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="56" spans="1:19" s="19" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A56" s="17" t="s">
-        <v>55</v>
-      </c>
-      <c r="B56" s="18"/>
-      <c r="F56" s="18">
-        <v>0</v>
-      </c>
-      <c r="G56" s="19">
-        <v>1</v>
-      </c>
-      <c r="H56" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="I56" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="T55" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="U55" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="V55" s="6" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="56" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A56" s="23" t="s">
+        <v>53</v>
+      </c>
+      <c r="E56" s="23"/>
+      <c r="F56">
+        <v>0</v>
+      </c>
+      <c r="G56">
+        <v>1</v>
+      </c>
+      <c r="H56" t="s">
+        <v>20</v>
+      </c>
+      <c r="I56" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="J56" s="18">
-        <v>0</v>
-      </c>
-      <c r="L56" s="20" t="s">
+      <c r="J56">
+        <v>0</v>
+      </c>
+      <c r="L56" t="s">
         <v>10</v>
       </c>
-      <c r="M56" s="20" t="s">
+      <c r="M56" t="s">
+        <v>61</v>
+      </c>
+      <c r="N56">
+        <v>1</v>
+      </c>
+      <c r="O56" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="N56" s="20">
-        <v>1</v>
-      </c>
-      <c r="O56" s="21" t="s">
-        <v>69</v>
-      </c>
-      <c r="P56" s="20" t="s">
+      <c r="P56" t="s">
         <v>17</v>
       </c>
-      <c r="Q56" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="R56" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="S56" s="20" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="57" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="Q56" t="s">
+        <v>20</v>
+      </c>
+      <c r="R56" t="s">
+        <v>68</v>
+      </c>
+      <c r="S56" t="s">
+        <v>76</v>
+      </c>
+      <c r="T56" t="s">
+        <v>87</v>
+      </c>
+      <c r="U56" t="s">
+        <v>86</v>
+      </c>
+      <c r="V56" s="17" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="57" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A57" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B57" s="1"/>
       <c r="C57" s="2"/>
@@ -2863,19 +3180,19 @@
         <v>10</v>
       </c>
       <c r="J57" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L57" s="5" t="s">
         <v>10</v>
       </c>
       <c r="M57" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="N57" s="2">
+        <v>1</v>
+      </c>
+      <c r="O57" s="7" t="s">
         <v>65</v>
-      </c>
-      <c r="N57" s="2">
-        <v>1</v>
-      </c>
-      <c r="O57" t="s">
-        <v>69</v>
       </c>
       <c r="P57" s="13" t="s">
         <v>17</v>
@@ -2884,166 +3201,250 @@
         <v>20</v>
       </c>
       <c r="R57" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="S57" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="S57" s="13" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="58" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A58" s="10"/>
-      <c r="B58" s="11"/>
-      <c r="C58" s="9"/>
-      <c r="D58" s="9"/>
-      <c r="E58" s="9"/>
-      <c r="F58" s="11"/>
-      <c r="G58" s="9"/>
-      <c r="H58" s="9"/>
-      <c r="I58" s="9"/>
-      <c r="J58" s="11"/>
-      <c r="K58" s="10"/>
-      <c r="L58" s="10"/>
-      <c r="M58" s="10"/>
-      <c r="N58" s="10"/>
-      <c r="O58" s="12"/>
-      <c r="P58" s="10"/>
-      <c r="Q58" s="10"/>
-      <c r="R58" s="9"/>
-      <c r="S58" s="9"/>
-    </row>
-    <row r="59" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A59" s="3" t="s">
+      <c r="T57" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="U57" s="13"/>
+      <c r="V57" s="18" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="58" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A58" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B58" s="1"/>
+      <c r="C58" s="2"/>
+      <c r="D58" s="2"/>
+      <c r="E58" s="2"/>
+      <c r="F58" s="1">
+        <v>0</v>
+      </c>
+      <c r="G58">
+        <v>1</v>
+      </c>
+      <c r="H58" t="s">
+        <v>20</v>
+      </c>
+      <c r="I58" t="s">
+        <v>10</v>
+      </c>
+      <c r="J58" s="1">
+        <v>1</v>
+      </c>
+      <c r="L58" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="M58" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="N58" s="2">
+        <v>1</v>
+      </c>
+      <c r="O58" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="P58" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q58" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="R58" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="S58" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="T58" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="U58" s="5"/>
+      <c r="V58" s="17" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="59" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A59" s="10"/>
+      <c r="B59" s="11"/>
+      <c r="C59" s="9"/>
+      <c r="D59" s="9"/>
+      <c r="E59" s="9"/>
+      <c r="F59" s="11"/>
+      <c r="G59" s="9"/>
+      <c r="H59" s="9"/>
+      <c r="I59" s="9"/>
+      <c r="J59" s="11"/>
+      <c r="K59" s="10"/>
+      <c r="L59" s="10"/>
+      <c r="M59" s="10"/>
+      <c r="N59" s="10"/>
+      <c r="O59" s="12"/>
+      <c r="P59" s="10"/>
+      <c r="Q59" s="10"/>
+      <c r="R59" s="9"/>
+      <c r="S59" s="9"/>
+      <c r="T59" s="9"/>
+      <c r="U59" s="9"/>
+      <c r="V59" s="9"/>
+    </row>
+    <row r="60" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A60" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B59" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="C59" s="3"/>
-      <c r="D59" s="3"/>
-      <c r="E59" s="3"/>
-      <c r="F59" s="4" t="s">
+      <c r="B60" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C60" s="3"/>
+      <c r="D60" s="3"/>
+      <c r="E60" s="3"/>
+      <c r="F60" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="G59" s="3"/>
-      <c r="H59" s="3"/>
-      <c r="I59" s="3"/>
-      <c r="J59" s="4" t="s">
+      <c r="G60" s="3"/>
+      <c r="H60" s="3"/>
+      <c r="I60" s="3"/>
+      <c r="J60" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="K59" s="3"/>
-      <c r="L59" s="3"/>
-      <c r="M59" s="3"/>
-      <c r="N59" s="3"/>
-      <c r="O59" s="8"/>
-      <c r="P59" s="3" t="s">
+      <c r="K60" s="3"/>
+      <c r="L60" s="3"/>
+      <c r="M60" s="3"/>
+      <c r="N60" s="3"/>
+      <c r="O60" s="8"/>
+      <c r="P60" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="Q59" s="3"/>
-      <c r="R59" s="3"/>
-      <c r="S59" s="3"/>
-    </row>
-    <row r="60" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A60" s="9" t="s">
+      <c r="Q60" s="3"/>
+      <c r="R60" s="3"/>
+      <c r="S60" s="3"/>
+      <c r="T60" s="3"/>
+      <c r="U60" s="3"/>
+      <c r="V60" s="3"/>
+    </row>
+    <row r="61" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A61" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="B61" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C61" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="D61" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="E61" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="F61" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="G61" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="H61" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="I61" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="J61" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="K61" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="L61" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="M61" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="N61" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="O61" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="P61" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q61" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="R61" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="S61" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="T61" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="U61" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="B60" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="C60" s="9" t="s">
-        <v>2</v>
-      </c>
-      <c r="D60" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="E60" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="F60" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="G60" s="9" t="s">
-        <v>2</v>
-      </c>
-      <c r="H60" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="I60" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="J60" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="K60" s="9" t="s">
-        <v>2</v>
-      </c>
-      <c r="L60" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="M60" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="N60" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="O60" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="P60" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q60" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="R60" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="S60" s="6" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="61" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A61" s="14" t="s">
-        <v>48</v>
-      </c>
-      <c r="B61" s="1"/>
-      <c r="F61" s="1">
-        <v>0</v>
-      </c>
-      <c r="G61">
-        <v>1</v>
-      </c>
-      <c r="H61" t="s">
-        <v>20</v>
-      </c>
-      <c r="I61" t="s">
+      <c r="V61" s="6" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="62" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A62" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="B62" s="1"/>
+      <c r="F62" s="1">
+        <v>0</v>
+      </c>
+      <c r="G62">
+        <v>1</v>
+      </c>
+      <c r="H62" t="s">
+        <v>20</v>
+      </c>
+      <c r="I62" t="s">
         <v>10</v>
       </c>
-      <c r="J61" s="1">
-        <v>0</v>
-      </c>
-      <c r="L61" s="5" t="s">
+      <c r="J62" s="1">
+        <v>0</v>
+      </c>
+      <c r="L62" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="M61" s="2" t="s">
+      <c r="M62" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="N62" s="2">
+        <v>1</v>
+      </c>
+      <c r="O62" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="N61" s="2">
-        <v>1</v>
-      </c>
-      <c r="O61" t="s">
-        <v>69</v>
-      </c>
-      <c r="P61" s="5" t="s">
+      <c r="P62" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="Q61" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="R61" s="13" t="s">
+      <c r="Q62" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="R62" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="S62" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="S61" s="13" t="s">
-        <v>77</v>
+      <c r="T62" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="U62" s="13"/>
+      <c r="V62" s="18" t="s">
+        <v>90</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
just one more test
</commit_message>
<xml_diff>
--- a/examples/scripts/test_pv.xlsx
+++ b/examples/scripts/test_pv.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="555" uniqueCount="96">
   <si>
     <t>dispatchable</t>
   </si>
@@ -306,6 +306,12 @@
   </si>
   <si>
     <t>pv_capacity below real peak capacity of 0.135 kWp, but real peak capacity could be accessed separately</t>
+  </si>
+  <si>
+    <t>_dispfix_pv_fix</t>
+  </si>
+  <si>
+    <t>for pv-panel-8, disp with profile can also be used instead of vol…all previous configurations where profiles were scaled down or cut off should work with this panel. Maybe add extra excess for volatile.</t>
   </si>
 </sst>
 </file>
@@ -788,7 +794,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:V62"/>
+  <dimension ref="A1:V63"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.08984375" customWidth="1"/>
@@ -3270,180 +3276,225 @@
       </c>
     </row>
     <row r="59" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A59" s="10"/>
-      <c r="B59" s="11"/>
-      <c r="C59" s="9"/>
-      <c r="D59" s="9"/>
-      <c r="E59" s="9"/>
-      <c r="F59" s="11"/>
-      <c r="G59" s="9"/>
-      <c r="H59" s="9"/>
-      <c r="I59" s="9"/>
-      <c r="J59" s="11"/>
-      <c r="K59" s="10"/>
-      <c r="L59" s="10"/>
-      <c r="M59" s="10"/>
-      <c r="N59" s="10"/>
-      <c r="O59" s="12"/>
-      <c r="P59" s="10"/>
-      <c r="Q59" s="10"/>
-      <c r="R59" s="9"/>
-      <c r="S59" s="9"/>
-      <c r="T59" s="9"/>
-      <c r="U59" s="9"/>
-      <c r="V59" s="9"/>
+      <c r="A59" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="B59" s="1">
+        <v>1</v>
+      </c>
+      <c r="C59" s="2"/>
+      <c r="D59" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E59" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F59" s="1"/>
+      <c r="J59" s="1">
+        <v>1</v>
+      </c>
+      <c r="L59" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="M59" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="N59" s="2">
+        <v>1</v>
+      </c>
+      <c r="O59" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="P59" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q59" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="R59" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="S59" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="T59" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="U59" s="5"/>
+      <c r="V59" s="17" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="60" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A60" s="3" t="s">
+      <c r="A60" s="5"/>
+      <c r="B60" s="1"/>
+      <c r="C60" s="2"/>
+      <c r="D60" s="2"/>
+      <c r="E60" s="2"/>
+      <c r="F60" s="1"/>
+      <c r="J60" s="1"/>
+      <c r="L60" s="2"/>
+      <c r="M60" s="2"/>
+      <c r="N60" s="2"/>
+      <c r="O60" s="7"/>
+      <c r="P60" s="5"/>
+      <c r="Q60" s="5"/>
+      <c r="R60" s="5"/>
+      <c r="S60" s="5"/>
+      <c r="T60" s="5"/>
+      <c r="U60" s="5"/>
+    </row>
+    <row r="61" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A61" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B60" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="C60" s="3"/>
-      <c r="D60" s="3"/>
-      <c r="E60" s="3"/>
-      <c r="F60" s="4" t="s">
+      <c r="B61" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C61" s="3"/>
+      <c r="D61" s="3"/>
+      <c r="E61" s="3"/>
+      <c r="F61" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="G60" s="3"/>
-      <c r="H60" s="3"/>
-      <c r="I60" s="3"/>
-      <c r="J60" s="4" t="s">
+      <c r="G61" s="3"/>
+      <c r="H61" s="3"/>
+      <c r="I61" s="3"/>
+      <c r="J61" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="K60" s="3"/>
-      <c r="L60" s="3"/>
-      <c r="M60" s="3"/>
-      <c r="N60" s="3"/>
-      <c r="O60" s="8"/>
-      <c r="P60" s="3" t="s">
+      <c r="K61" s="3"/>
+      <c r="L61" s="3"/>
+      <c r="M61" s="3"/>
+      <c r="N61" s="3"/>
+      <c r="O61" s="8"/>
+      <c r="P61" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="Q60" s="3"/>
-      <c r="R60" s="3"/>
-      <c r="S60" s="3"/>
-      <c r="T60" s="3"/>
-      <c r="U60" s="3"/>
-      <c r="V60" s="3"/>
-    </row>
-    <row r="61" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A61" s="9" t="s">
+      <c r="Q61" s="3"/>
+      <c r="R61" s="3"/>
+      <c r="S61" s="3"/>
+      <c r="T61" s="3"/>
+      <c r="U61" s="3"/>
+      <c r="V61" s="3"/>
+    </row>
+    <row r="62" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A62" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="B61" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="C61" s="9" t="s">
+      <c r="B62" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C62" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D61" s="9" t="s">
+      <c r="D62" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="E61" s="9" t="s">
+      <c r="E62" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="F61" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="G61" s="9" t="s">
+      <c r="F62" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="G62" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="H61" s="9" t="s">
+      <c r="H62" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="I61" s="9" t="s">
+      <c r="I62" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="J61" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="K61" s="9" t="s">
+      <c r="J62" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="K62" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="L61" s="9" t="s">
+      <c r="L62" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="M61" s="9" t="s">
+      <c r="M62" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="N61" s="9" t="s">
+      <c r="N62" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="O61" s="12" t="s">
+      <c r="O62" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="P61" s="6" t="s">
+      <c r="P62" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="Q61" s="6" t="s">
+      <c r="Q62" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="R61" s="6" t="s">
+      <c r="R62" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="S61" s="6" t="s">
+      <c r="S62" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="T61" s="6" t="s">
+      <c r="T62" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="U61" s="6" t="s">
+      <c r="U62" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="V61" s="6" t="s">
+      <c r="V62" s="6" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="62" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A62" s="14" t="s">
+    <row r="63" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A63" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="B62" s="1"/>
-      <c r="F62" s="1">
-        <v>0</v>
-      </c>
-      <c r="G62">
-        <v>1</v>
-      </c>
-      <c r="H62" t="s">
-        <v>20</v>
-      </c>
-      <c r="I62" t="s">
+      <c r="B63" s="1"/>
+      <c r="F63" s="1">
+        <v>0</v>
+      </c>
+      <c r="G63">
+        <v>1</v>
+      </c>
+      <c r="H63" t="s">
+        <v>20</v>
+      </c>
+      <c r="I63" t="s">
         <v>10</v>
       </c>
-      <c r="J62" s="1">
-        <v>0</v>
-      </c>
-      <c r="L62" s="5" t="s">
+      <c r="J63" s="1">
+        <v>0</v>
+      </c>
+      <c r="L63" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="M62" s="2" t="s">
+      <c r="M63" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="N62" s="2">
-        <v>1</v>
-      </c>
-      <c r="O62" s="8" t="s">
+      <c r="N63" s="2">
+        <v>1</v>
+      </c>
+      <c r="O63" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="P62" s="5" t="s">
+      <c r="P63" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="Q62" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="R62" s="13" t="s">
+      <c r="Q63" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="R63" s="13" t="s">
         <v>68</v>
       </c>
-      <c r="S62" s="13" t="s">
+      <c r="S63" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="T62" s="13" t="s">
+      <c r="T63" s="13" t="s">
         <v>88</v>
       </c>
-      <c r="U62" s="13"/>
-      <c r="V62" s="18" t="s">
+      <c r="U63" s="13"/>
+      <c r="V63" s="18" t="s">
         <v>90</v>
       </c>
     </row>

</xml_diff>